<commit_message>
updates to NNT table
</commit_message>
<xml_diff>
--- a/results/result-tables-13feb2024_v2.xlsx
+++ b/results/result-tables-13feb2024_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mgarc48\git\COVID-Corporate\COVID-Corporate\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4268D47-8DDE-477F-985C-9276029757C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C6ED62-65E5-4AAD-95B9-6917AA0DC81B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-2085" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6262,12 +6262,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="74">
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -6676,6 +6670,12 @@
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -6690,102 +6690,102 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EB39D523-8CE6-467A-8BF2-0943F09CD9AA}" name="Table1" displayName="Table1" ref="A1:Q71" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EB39D523-8CE6-467A-8BF2-0943F09CD9AA}" name="Table1" displayName="Table1" ref="A1:Q71" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
   <autoFilter ref="A1:Q71" xr:uid="{EB39D523-8CE6-467A-8BF2-0943F09CD9AA}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{11DF3030-1E48-4CE9-8C3E-6BFCB987473B}" name="scenario" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{0BC45011-D64B-496E-94EC-7EE280EDD54B}" name="IsoMild" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{C504D3CC-0A0B-4178-AD62-CBDEFC582D06}" name="IsoSevere" dataDxfId="71"/>
-    <tableColumn id="4" xr3:uid="{BF03DDEC-1F0E-4425-A5E0-7A0C6B519069}" name="PostIsoMask" dataDxfId="70"/>
-    <tableColumn id="5" xr3:uid="{903DBAF9-91AB-49F5-9976-7F0EED85B049}" name="ExpMask" dataDxfId="69"/>
-    <tableColumn id="6" xr3:uid="{CBEAA386-C470-499F-B013-9CF2286B8492}" name="IsoEnd" dataDxfId="68"/>
-    <tableColumn id="7" xr3:uid="{1387EA39-66D6-4130-B7E7-98C2A8C31536}" name="IsoMildWork" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{59ADFE0E-088A-4CF2-AF33-5CD1639A447A}" name="IsoSevereWork" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{6D9CEDF6-94CA-4D98-B640-506324BB5A9F}" name="PostIsoMaskWork" dataDxfId="65"/>
-    <tableColumn id="10" xr3:uid="{F22D7D50-3B32-4B17-85F6-4DFC96C4A520}" name="ExpMaskWork" dataDxfId="64"/>
-    <tableColumn id="11" xr3:uid="{7E06DF55-C593-4C2E-8C9E-1A0576DCC334}" name="IsoEndWork" dataDxfId="63"/>
-    <tableColumn id="12" xr3:uid="{CCBEF845-9B22-422F-8476-4FE2D61DEE82}" name="iso.prob.x" dataDxfId="62"/>
-    <tableColumn id="13" xr3:uid="{E2D6CBFA-4CF2-4233-9DD7-06107D592A7C}" name="notif.work" dataDxfId="61"/>
-    <tableColumn id="14" xr3:uid="{7E33EA16-10A0-4A56-B342-87A78EBFE672}" name="notif.com" dataDxfId="60"/>
-    <tableColumn id="15" xr3:uid="{DAB9DFD0-11DD-4E40-A42A-567BB7671627}" name="notif.home" dataDxfId="59"/>
-    <tableColumn id="16" xr3:uid="{1764A1B0-D5EC-465E-B29C-EB05CA4C0DBC}" name="act.rate.iso" dataDxfId="58"/>
-    <tableColumn id="17" xr3:uid="{A86517B1-6943-46AE-93EF-BECF2E0C413F}" name="inf.prob.mask" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{11DF3030-1E48-4CE9-8C3E-6BFCB987473B}" name="scenario" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{0BC45011-D64B-496E-94EC-7EE280EDD54B}" name="IsoMild" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{C504D3CC-0A0B-4178-AD62-CBDEFC582D06}" name="IsoSevere" dataDxfId="69"/>
+    <tableColumn id="4" xr3:uid="{BF03DDEC-1F0E-4425-A5E0-7A0C6B519069}" name="PostIsoMask" dataDxfId="68"/>
+    <tableColumn id="5" xr3:uid="{903DBAF9-91AB-49F5-9976-7F0EED85B049}" name="ExpMask" dataDxfId="67"/>
+    <tableColumn id="6" xr3:uid="{CBEAA386-C470-499F-B013-9CF2286B8492}" name="IsoEnd" dataDxfId="66"/>
+    <tableColumn id="7" xr3:uid="{1387EA39-66D6-4130-B7E7-98C2A8C31536}" name="IsoMildWork" dataDxfId="65"/>
+    <tableColumn id="8" xr3:uid="{59ADFE0E-088A-4CF2-AF33-5CD1639A447A}" name="IsoSevereWork" dataDxfId="64"/>
+    <tableColumn id="9" xr3:uid="{6D9CEDF6-94CA-4D98-B640-506324BB5A9F}" name="PostIsoMaskWork" dataDxfId="63"/>
+    <tableColumn id="10" xr3:uid="{F22D7D50-3B32-4B17-85F6-4DFC96C4A520}" name="ExpMaskWork" dataDxfId="62"/>
+    <tableColumn id="11" xr3:uid="{7E06DF55-C593-4C2E-8C9E-1A0576DCC334}" name="IsoEndWork" dataDxfId="61"/>
+    <tableColumn id="12" xr3:uid="{CCBEF845-9B22-422F-8476-4FE2D61DEE82}" name="iso.prob.x" dataDxfId="60"/>
+    <tableColumn id="13" xr3:uid="{E2D6CBFA-4CF2-4233-9DD7-06107D592A7C}" name="notif.work" dataDxfId="59"/>
+    <tableColumn id="14" xr3:uid="{7E33EA16-10A0-4A56-B342-87A78EBFE672}" name="notif.com" dataDxfId="58"/>
+    <tableColumn id="15" xr3:uid="{DAB9DFD0-11DD-4E40-A42A-567BB7671627}" name="notif.home" dataDxfId="57"/>
+    <tableColumn id="16" xr3:uid="{1764A1B0-D5EC-465E-B29C-EB05CA4C0DBC}" name="act.rate.iso" dataDxfId="56"/>
+    <tableColumn id="17" xr3:uid="{A86517B1-6943-46AE-93EF-BECF2E0C413F}" name="inf.prob.mask" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{55487487-76E1-43D3-AD7C-D8406C6232F3}" name="Table2" displayName="Table2" ref="A1:Q71" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{55487487-76E1-43D3-AD7C-D8406C6232F3}" name="Table2" displayName="Table2" ref="A1:Q71" totalsRowShown="0" headerRowDxfId="54" dataDxfId="53">
   <autoFilter ref="A1:Q71" xr:uid="{55487487-76E1-43D3-AD7C-D8406C6232F3}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{A6BD61E2-9F79-42B6-8CC6-DD8D57E80A0A}" name="scenario" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{E8B0F682-689B-488E-8D9E-FF33367FB502}" name="CInc" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{4114E6CC-F7E9-434B-B376-6DAD59990ED0}" name="IncAverted" dataDxfId="52"/>
-    <tableColumn id="4" xr3:uid="{E0C8854F-6A61-4E93-B556-5F5842AEEF6F}" name="PctAverted" dataDxfId="51"/>
-    <tableColumn id="5" xr3:uid="{34508F3B-243C-4545-9D21-596EC281D5D3}" name="AvertedPerIso" dataDxfId="50"/>
-    <tableColumn id="6" xr3:uid="{FB2CDA87-3863-4CD0-B97E-A1792F21AB8A}" name="NNT" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{132B1188-463E-4744-BC1A-71A06C12A997}" name="CIncWork" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{DFDD86D0-CE98-4EAE-AC6A-825AB4369A2F}" name="IncAvertedWork" dataDxfId="47"/>
-    <tableColumn id="9" xr3:uid="{96001940-73AE-4E4D-B003-3E0ACE8A0255}" name="PctAvertedWork" dataDxfId="46"/>
-    <tableColumn id="10" xr3:uid="{4E64A19A-D89C-40D6-87B1-8203C69AA38A}" name="AvertedPerIsoWork" dataDxfId="45"/>
-    <tableColumn id="11" xr3:uid="{D5C462E9-DEB7-481A-AF19-E2BE63E06EBC}" name="NNTWork" dataDxfId="44"/>
-    <tableColumn id="12" xr3:uid="{736D657B-25F1-4041-9C83-BB56050EA329}" name="iso.prob.x" dataDxfId="43"/>
-    <tableColumn id="13" xr3:uid="{0CCA4132-2319-4403-9E2A-E688F1438B2E}" name="notif.work" dataDxfId="42"/>
-    <tableColumn id="14" xr3:uid="{EF2E8CE9-A7FC-46EF-AD0F-BC03A9F4377D}" name="notif.com" dataDxfId="41"/>
-    <tableColumn id="15" xr3:uid="{503FDF13-F551-41B9-9382-30886B513090}" name="notif.home" dataDxfId="40"/>
-    <tableColumn id="16" xr3:uid="{E42CFF88-4768-4585-B095-8376AFCC0BF1}" name="act.rate.iso" dataDxfId="39"/>
-    <tableColumn id="17" xr3:uid="{B1E03A32-15A3-4015-861D-D0F2A90C41D5}" name="inf.prob.mask" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{A6BD61E2-9F79-42B6-8CC6-DD8D57E80A0A}" name="scenario" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{E8B0F682-689B-488E-8D9E-FF33367FB502}" name="CInc" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{4114E6CC-F7E9-434B-B376-6DAD59990ED0}" name="IncAverted" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{E0C8854F-6A61-4E93-B556-5F5842AEEF6F}" name="PctAverted" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{34508F3B-243C-4545-9D21-596EC281D5D3}" name="AvertedPerIso" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{FB2CDA87-3863-4CD0-B97E-A1792F21AB8A}" name="NNT" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{132B1188-463E-4744-BC1A-71A06C12A997}" name="CIncWork" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{DFDD86D0-CE98-4EAE-AC6A-825AB4369A2F}" name="IncAvertedWork" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{96001940-73AE-4E4D-B003-3E0ACE8A0255}" name="PctAvertedWork" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{4E64A19A-D89C-40D6-87B1-8203C69AA38A}" name="AvertedPerIsoWork" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{D5C462E9-DEB7-481A-AF19-E2BE63E06EBC}" name="NNTWork" dataDxfId="42"/>
+    <tableColumn id="12" xr3:uid="{736D657B-25F1-4041-9C83-BB56050EA329}" name="iso.prob.x" dataDxfId="41"/>
+    <tableColumn id="13" xr3:uid="{0CCA4132-2319-4403-9E2A-E688F1438B2E}" name="notif.work" dataDxfId="40"/>
+    <tableColumn id="14" xr3:uid="{EF2E8CE9-A7FC-46EF-AD0F-BC03A9F4377D}" name="notif.com" dataDxfId="39"/>
+    <tableColumn id="15" xr3:uid="{503FDF13-F551-41B9-9382-30886B513090}" name="notif.home" dataDxfId="38"/>
+    <tableColumn id="16" xr3:uid="{E42CFF88-4768-4585-B095-8376AFCC0BF1}" name="act.rate.iso" dataDxfId="37"/>
+    <tableColumn id="17" xr3:uid="{B1E03A32-15A3-4015-861D-D0F2A90C41D5}" name="inf.prob.mask" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A3898F9C-6180-415E-BFD5-5BEDE863BE19}" name="Table3" displayName="Table3" ref="A1:O71" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A3898F9C-6180-415E-BFD5-5BEDE863BE19}" name="Table3" displayName="Table3" ref="A1:O71" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="A1:O71" xr:uid="{A3898F9C-6180-415E-BFD5-5BEDE863BE19}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{44659A06-10D2-4DE9-BDBB-9D77ECCCCBBA}" name="scenario" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{AD453684-E89C-457E-8478-30E0FE70EEFC}" name="CDeaths" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{93CE2EFA-AE0F-4A77-B970-3670B80CC45A}" name="DeathsAverted" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{1280A413-8902-4326-A381-94E26E1AF998}" name="PctAverted" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{3CAF910E-3334-4EA5-B044-F00F47DF55F9}" name="AvertedPerIso" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{4F91718A-C856-42C7-B674-DC1CD541828C}" name="CDeathsWork" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{075BD288-1406-498B-ABF2-D529C1686500}" name="DeathsAvertedWork" dataDxfId="29"/>
-    <tableColumn id="8" xr3:uid="{F5B9B652-8085-4744-9578-57C748256C78}" name="PctAvertedWork" dataDxfId="28"/>
-    <tableColumn id="9" xr3:uid="{7F1C77BA-2C9B-4191-9122-D2C01A6A629D}" name="AvertedPerIsoWork" dataDxfId="27"/>
-    <tableColumn id="10" xr3:uid="{0378DA82-57A3-4F6D-8D1A-585C2B40130B}" name="iso.prob.x" dataDxfId="26"/>
-    <tableColumn id="11" xr3:uid="{489B494E-B433-4F80-9733-88DCC97F95BE}" name="notif.work" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{4DE17764-6B9A-494A-839F-CCC71F5F7447}" name="notif.com" dataDxfId="24"/>
-    <tableColumn id="13" xr3:uid="{A3A0165A-25AA-4306-BA7D-A3F08F41D26F}" name="notif.home" dataDxfId="23"/>
-    <tableColumn id="14" xr3:uid="{70A2A327-A03F-49A7-A252-8117F3AA7746}" name="act.rate.iso" dataDxfId="22"/>
-    <tableColumn id="15" xr3:uid="{D1AFC785-7186-4908-92B0-A97ACE4FAC06}" name="inf.prob.mask" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{44659A06-10D2-4DE9-BDBB-9D77ECCCCBBA}" name="scenario" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{AD453684-E89C-457E-8478-30E0FE70EEFC}" name="CDeaths" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{93CE2EFA-AE0F-4A77-B970-3670B80CC45A}" name="DeathsAverted" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{1280A413-8902-4326-A381-94E26E1AF998}" name="PctAverted" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{3CAF910E-3334-4EA5-B044-F00F47DF55F9}" name="AvertedPerIso" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{4F91718A-C856-42C7-B674-DC1CD541828C}" name="CDeathsWork" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{075BD288-1406-498B-ABF2-D529C1686500}" name="DeathsAvertedWork" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{F5B9B652-8085-4744-9578-57C748256C78}" name="PctAvertedWork" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{7F1C77BA-2C9B-4191-9122-D2C01A6A629D}" name="AvertedPerIsoWork" dataDxfId="25"/>
+    <tableColumn id="10" xr3:uid="{0378DA82-57A3-4F6D-8D1A-585C2B40130B}" name="iso.prob.x" dataDxfId="24"/>
+    <tableColumn id="11" xr3:uid="{489B494E-B433-4F80-9733-88DCC97F95BE}" name="notif.work" dataDxfId="23"/>
+    <tableColumn id="12" xr3:uid="{4DE17764-6B9A-494A-839F-CCC71F5F7447}" name="notif.com" dataDxfId="22"/>
+    <tableColumn id="13" xr3:uid="{A3A0165A-25AA-4306-BA7D-A3F08F41D26F}" name="notif.home" dataDxfId="21"/>
+    <tableColumn id="14" xr3:uid="{70A2A327-A03F-49A7-A252-8117F3AA7746}" name="act.rate.iso" dataDxfId="20"/>
+    <tableColumn id="15" xr3:uid="{D1AFC785-7186-4908-92B0-A97ACE4FAC06}" name="inf.prob.mask" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7DDAF46C-14AF-4DAA-83AF-CB98D9166932}" name="Table4" displayName="Table4" ref="A1:Q71" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7DDAF46C-14AF-4DAA-83AF-CB98D9166932}" name="Table4" displayName="Table4" ref="A1:Q71" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A1:Q71" xr:uid="{7DDAF46C-14AF-4DAA-83AF-CB98D9166932}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{4FDCCE16-6562-49E4-8175-A5A58CBCC4EC}" name="scenario" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{629C4638-DC92-4250-AA77-B563412FE438}" name="CCase" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{E8D744BA-BE7F-4268-8125-6A07274D3F6B}" name="CaseAverted" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{8731EF8D-5EEA-421F-A1AA-D1FCDEFDE645}" name="PctAverted" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{BBF9A80E-7175-4446-8E07-08BDF3364962}" name="AvertedPerIso" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{51B4B640-F84F-46D4-8D7B-5A1C3B510159}" name="NNT" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{235FCB9E-CC40-4B99-B66A-0ADC0F98F87B}" name="CCaseWork" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{AC84C3F8-DFAE-479E-89E9-C92D0BFEF629}" name="CaseAvertedWork" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{9A89F3BA-33C3-4A00-A1CC-B639E819832D}" name="PctAvertedWork" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{55560A09-E6F6-4F95-ABE9-D555B0033610}" name="AvertedPerIsoWork" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{2242D241-AD9F-460C-9BC1-CD80C53CE6F4}" name="NNTWork" dataDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{C7131CED-1FBD-443C-88D1-24E037181889}" name="iso.prob.x" dataDxfId="7"/>
-    <tableColumn id="13" xr3:uid="{C967D3A9-5E1F-422B-AAAD-03B45498D720}" name="notif.work" dataDxfId="6"/>
-    <tableColumn id="14" xr3:uid="{CEA8EBD4-1010-4A9C-B548-9A6F85B9BD1C}" name="notif.com" dataDxfId="5"/>
-    <tableColumn id="15" xr3:uid="{A4F82A2C-3B5E-43EF-BCD2-CBFEB8CE43D4}" name="notif.home" dataDxfId="4"/>
-    <tableColumn id="16" xr3:uid="{720ED698-01D2-4820-9501-EB7B1FF1EAFC}" name="act.rate.iso" dataDxfId="3"/>
-    <tableColumn id="17" xr3:uid="{2CF451F9-244C-43DA-A83D-6722AF14439A}" name="inf.prob.mask" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{4FDCCE16-6562-49E4-8175-A5A58CBCC4EC}" name="scenario" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{629C4638-DC92-4250-AA77-B563412FE438}" name="CCase" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{E8D744BA-BE7F-4268-8125-6A07274D3F6B}" name="CaseAverted" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{8731EF8D-5EEA-421F-A1AA-D1FCDEFDE645}" name="PctAverted" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{BBF9A80E-7175-4446-8E07-08BDF3364962}" name="AvertedPerIso" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{51B4B640-F84F-46D4-8D7B-5A1C3B510159}" name="NNT" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{235FCB9E-CC40-4B99-B66A-0ADC0F98F87B}" name="CCaseWork" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{AC84C3F8-DFAE-479E-89E9-C92D0BFEF629}" name="CaseAvertedWork" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{9A89F3BA-33C3-4A00-A1CC-B639E819832D}" name="PctAvertedWork" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{55560A09-E6F6-4F95-ABE9-D555B0033610}" name="AvertedPerIsoWork" dataDxfId="7"/>
+    <tableColumn id="11" xr3:uid="{2242D241-AD9F-460C-9BC1-CD80C53CE6F4}" name="NNTWork" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{C7131CED-1FBD-443C-88D1-24E037181889}" name="iso.prob.x" dataDxfId="5"/>
+    <tableColumn id="13" xr3:uid="{C967D3A9-5E1F-422B-AAAD-03B45498D720}" name="notif.work" dataDxfId="4"/>
+    <tableColumn id="14" xr3:uid="{CEA8EBD4-1010-4A9C-B548-9A6F85B9BD1C}" name="notif.com" dataDxfId="3"/>
+    <tableColumn id="15" xr3:uid="{A4F82A2C-3B5E-43EF-BCD2-CBFEB8CE43D4}" name="notif.home" dataDxfId="2"/>
+    <tableColumn id="16" xr3:uid="{720ED698-01D2-4820-9501-EB7B1FF1EAFC}" name="act.rate.iso" dataDxfId="1"/>
+    <tableColumn id="17" xr3:uid="{2CF451F9-244C-43DA-A83D-6722AF14439A}" name="inf.prob.mask" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>